<commit_message>
feat(inventory): add confirmation alerts before stock adjustments
</commit_message>
<xml_diff>
--- a/REQUIREMENTS_TRACEABILITY_MATRIX.xlsx
+++ b/REQUIREMENTS_TRACEABILITY_MATRIX.xlsx
@@ -648,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -692,27 +692,27 @@
     <row r="5">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>62
+          <t>71
 TOTAL REQUIREMENTS</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>28
+          <t>33
 FUNCTIONAL REQS (FR)</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>21
+          <t>24
 NON-FUNCTIONAL (NFR)</t>
         </is>
       </c>
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>7
+          <t>14
 STAKEHOLDER NEEDS</t>
         </is>
       </c>
@@ -813,12 +813,12 @@
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>Screen 1 (POS Scan)</t>
+          <t>Screen 1 (POS Scan) &amp; Screen 3</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Jest, Camera Simulator, Haptics</t>
+          <t>Jest, Camera Simulator, Held Carts</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
@@ -839,11 +839,11 @@
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>5 Must / 0 Should</t>
+          <t>6 Must / 1 Should</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Atomic SQLite Tests, ViewShot</t>
+          <t>Atomic SQLite Tests, ViewShot, Bluetooth ESC/POS</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
@@ -874,11 +874,11 @@
         </is>
       </c>
       <c r="D14" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>4 Must / 0 Should</t>
+          <t>5 Must / 0 Should</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Modulo-10 Checksum Tests</t>
+          <t>Modulo-10 Checksum Tests, FEFO Expiry</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
@@ -1045,25 +1045,25 @@
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>Store Settings &amp; Local Backup</t>
+          <t>Store Settings &amp; Security Access Control</t>
         </is>
       </c>
       <c r="D19" s="12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>3 Must / 0 Should</t>
+          <t>4 Must / 0 Should</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Screen 7 (Settings)</t>
+          <t>Screen 7 (Settings) &amp; PIN Modal</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>PRAGMA Checkpoint &amp; Share Sheet</t>
+          <t>PRAGMA Checkpoint, Salted SHA-256 PIN</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
@@ -1075,30 +1075,30 @@
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>NFR-P</t>
+          <t>MOD-9</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Performance Efficiency &amp; Latency</t>
+          <t>Sales History &amp; Profit Intelligence</t>
         </is>
       </c>
       <c r="D20" s="10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>6 Must / 0 Should</t>
+          <t>1 Must / 0 Should</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
-          <t>Cross-Cutting</t>
+          <t>Screen 5 (Sales History)</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Android Systrace, adb start -W</t>
+          <t>Snapshot COGS, Tubo Formula, Privacy Mask</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
@@ -1110,30 +1110,30 @@
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>NFR-R</t>
+          <t>NFR-P</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>Reliability &amp; Offline Autonomy</t>
+          <t>Performance Efficiency &amp; Latency</t>
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>4 Must / 0 Should</t>
+          <t>6 Must / 0 Should</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Local SQLite Architecture</t>
+          <t>Cross-Cutting</t>
         </is>
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>Network Isolation &amp; Crash Kill Tests</t>
+          <t>Android Systrace, adb start -W</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
@@ -1145,30 +1145,30 @@
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>NFR-U</t>
+          <t>NFR-R</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Usability &amp; Touch Ergonomics</t>
+          <t>Reliability &amp; Offline Autonomy</t>
         </is>
       </c>
       <c r="D22" s="10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>6 Must / 0 Should</t>
+          <t>4 Must / 0 Should</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>All 7 Screens</t>
+          <t>Local SQLite Architecture</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>WCAG Contrast, Accessibility Scanner</t>
+          <t>Network Isolation &amp; Crash Kill Tests</t>
         </is>
       </c>
       <c r="H22" s="10" t="inlineStr">
@@ -1180,30 +1180,30 @@
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>NFR-S</t>
+          <t>NFR-U</t>
         </is>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>Security, Privacy &amp; Audit Integrity</t>
+          <t>Usability &amp; Touch Ergonomics</t>
         </is>
       </c>
       <c r="D23" s="12" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>4 Must / 0 Should</t>
+          <t>6 Must / 0 Should</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Local Sandbox Storage</t>
+          <t>All 7 Screens</t>
         </is>
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>SQL Injection Fuzzing, PII Audit</t>
+          <t>WCAG Contrast, Multi-Dialect i18n</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
@@ -1215,30 +1215,30 @@
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>NFR-A</t>
+          <t>NFR-S</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Maintainability &amp; Code Architecture</t>
+          <t>Security, Privacy &amp; Audit Integrity</t>
         </is>
       </c>
       <c r="D24" s="10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>3 Must / 0 Should</t>
+          <t>6 Must / 0 Should</t>
         </is>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Domain / App / Infra</t>
+          <t>Local Sandbox Storage</t>
         </is>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>tsc --noEmit, Dependency Boundaries</t>
+          <t>SQL Injection Fuzzing, PIN Lockout, Privacy Masking</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
@@ -1250,33 +1250,68 @@
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="12" t="inlineStr">
         <is>
+          <t>NFR-A</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Maintainability &amp; Code Architecture</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>3 Must / 0 Should</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>Domain / App / Infra</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>tsc --noEmit, Dependency Boundaries</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="10" t="inlineStr">
+        <is>
           <t>NFR-E</t>
         </is>
       </c>
-      <c r="C25" s="13" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>Environmental &amp; Hardware Compatibility</t>
         </is>
       </c>
-      <c r="D25" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>2 Must / 0 Should</t>
-        </is>
-      </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="D26" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>3 Must / 0 Should</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>Android 10+ 2GB Devices</t>
         </is>
       </c>
-      <c r="G25" s="13" t="inlineStr">
-        <is>
-          <t>Thermal Sleep &amp; Low-RAM Profiling</t>
-        </is>
-      </c>
-      <c r="H25" s="12" t="inlineStr">
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>Thermal Sleep, AMOLED True-Black Battery Saver</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -1301,11 +1336,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M33"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
@@ -1671,27 +1706,27 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Cart Parking / Hold Basket (Park/Hold Cart)</t>
+          <t>Persistent Named Held Carts &amp; Multi-Customer Queue ("Stock" Basket)</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>SN-001</t>
+          <t>SN-001, SN-008</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>BG-001</t>
+          <t>BG-001, BG-008</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>BR-RUL-001</t>
-        </is>
-      </c>
-      <c r="G6" s="19" t="inlineStr">
-        <is>
-          <t>SHOULD</t>
+          <t>BR-RUL-007</t>
+        </is>
+      </c>
+      <c r="G6" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
@@ -1712,7 +1747,7 @@
       </c>
       <c r="K6" s="15" t="inlineStr">
         <is>
-          <t>Unit Test (Hold and Resume Basket)</t>
+          <t>Unit Test (Queue Prompt, Multi-Cart Restore/Delete, Cold-Boot Hydration)</t>
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr">
@@ -2069,944 +2104,947 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
+          <t>FR-TND-006</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Tender &amp; Settlement</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>58mm/80mm ESC/POS Bluetooth Thermal Receipt Slip Printing</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>SN-013</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>BG-011</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>BR-RUL-012</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Screen 3 &amp; Screen 5</t>
+        </is>
+      </c>
+      <c r="I12" s="15" t="inlineStr">
+        <is>
+          <t>src/app/checkout.tsx
+src/app/sales.tsx</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>sales_transactions</t>
+        </is>
+      </c>
+      <c r="K12" s="15" t="inlineStr">
+        <is>
+          <t>Bluetooth ESC/POS Payload Format &amp; Print Latency Test</t>
+        </is>
+      </c>
+      <c r="L12" s="10" t="inlineStr">
+        <is>
+          <t>TC-FR-TND-006</t>
+        </is>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>FR-TND-007</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Tender &amp; Settlement</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Static QR Ph / GCash Digital Payment Verification &amp; Convenience Surcharge</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>SN-014</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>BG-012</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>BR-RUL-013</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Screen 3 (Checkout)</t>
+        </is>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
+        <is>
+          <t>src/app/checkout.tsx
+src/domain/value-objects/Money.ts</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>sales_transactions</t>
+        </is>
+      </c>
+      <c r="K13" s="18" t="inlineStr">
+        <is>
+          <t>QR Ph Verification &amp; Surcharge Ledger Calculation Test</t>
+        </is>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>TC-FR-TND-007</t>
+        </is>
+      </c>
+      <c r="M13" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
           <t>FR-INV-001</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Catalog &amp; Inventory</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>Product Onboarding with Barcode Verification &amp; Auto-Generation</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>SN-001</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>BG-001</t>
         </is>
       </c>
-      <c r="F12" s="10" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>BR-RUL-001</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="H14" s="10" t="inlineStr">
         <is>
           <t>Screen 4 (Inventory)</t>
         </is>
       </c>
-      <c r="I12" s="15" t="inlineStr">
+      <c r="I14" s="15" t="inlineStr">
         <is>
           <t>src/app/inventory.tsx
 src/domain/value-objects/Barcode.ts</t>
         </is>
       </c>
-      <c r="J12" s="10" t="inlineStr">
+      <c r="J14" s="10" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="K12" s="15" t="inlineStr">
+      <c r="K14" s="15" t="inlineStr">
         <is>
           <t>Unit Test (GS1 Checksum &amp; Auto Tingi Code)</t>
         </is>
       </c>
-      <c r="L12" s="10" t="inlineStr">
+      <c r="L14" s="10" t="inlineStr">
         <is>
           <t>TC-FR-INV-001</t>
         </is>
       </c>
-      <c r="M12" s="17" t="inlineStr">
+      <c r="M14" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>FR-INV-002</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Catalog &amp; Inventory</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Multi-Tier Selling Units &amp; Fractional Tingi Conversion</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>SN-001</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>BG-001</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>BR-RUL-001</t>
         </is>
       </c>
-      <c r="G13" s="16" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>Screen 4 &amp; Screen 3</t>
         </is>
       </c>
-      <c r="I13" s="18" t="inlineStr">
+      <c r="I15" s="18" t="inlineStr">
         <is>
           <t>src/domain/entities/Product.ts
 src/application/TindahanStoreService.ts</t>
         </is>
       </c>
-      <c r="J13" s="12" t="inlineStr">
+      <c r="J15" s="12" t="inlineStr">
         <is>
           <t>products (selling_tiers_json)</t>
         </is>
       </c>
-      <c r="K13" s="18" t="inlineStr">
+      <c r="K15" s="18" t="inlineStr">
         <is>
           <t>Unit Test (Piece, Pack, Case Stock Math)</t>
         </is>
       </c>
-      <c r="L13" s="12" t="inlineStr">
+      <c r="L15" s="12" t="inlineStr">
         <is>
           <t>TC-FR-INV-002</t>
         </is>
       </c>
-      <c r="M13" s="17" t="inlineStr">
+      <c r="M15" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>FR-INV-003</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Catalog &amp; Inventory</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>Reason-Coded Stock Adjustments (Delivery, Household, Spoilage, Audit)</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>SN-003</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>BG-003</t>
         </is>
       </c>
-      <c r="F14" s="10" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>BR-RUL-002</t>
         </is>
       </c>
-      <c r="G14" s="16" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="H16" s="10" t="inlineStr">
         <is>
           <t>Screen 4 (Inventory)</t>
         </is>
       </c>
-      <c r="I14" s="15" t="inlineStr">
+      <c r="I16" s="15" t="inlineStr">
         <is>
           <t>src/app/inventory.tsx
 src/application/TindahanStoreService.ts</t>
         </is>
       </c>
-      <c r="J14" s="10" t="inlineStr">
+      <c r="J16" s="10" t="inlineStr">
         <is>
           <t>products, shrinkage_logs</t>
         </is>
       </c>
-      <c r="K14" s="15" t="inlineStr">
+      <c r="K16" s="15" t="inlineStr">
         <is>
           <t>Integration Test (Audit Logs &amp; Ledger Entries)</t>
         </is>
       </c>
-      <c r="L14" s="10" t="inlineStr">
+      <c r="L16" s="10" t="inlineStr">
         <is>
           <t>TC-FR-INV-003</t>
         </is>
       </c>
-      <c r="M14" s="17" t="inlineStr">
+      <c r="M16" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>FR-INV-004</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Catalog &amp; Inventory</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>Triple-Encoded Stock Status Badges &amp; Dynamic Reorder Alerts</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>SN-006</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>BG-006</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr">
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>BR-RUL-001</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="H17" s="12" t="inlineStr">
         <is>
           <t>Screen 2 &amp; Screen 4</t>
         </is>
       </c>
-      <c r="I15" s="18" t="inlineStr">
+      <c r="I17" s="18" t="inlineStr">
         <is>
           <t>src/app/products.tsx
 src/app/inventory.tsx</t>
         </is>
       </c>
-      <c r="J15" s="12" t="inlineStr">
+      <c r="J17" s="12" t="inlineStr">
         <is>
           <t>products</t>
         </is>
       </c>
-      <c r="K15" s="18" t="inlineStr">
+      <c r="K17" s="18" t="inlineStr">
         <is>
           <t>Visual Regression &amp; Accessibility Test</t>
         </is>
       </c>
-      <c r="L15" s="12" t="inlineStr">
+      <c r="L17" s="12" t="inlineStr">
         <is>
           <t>TC-FR-INV-004</t>
         </is>
       </c>
-      <c r="M15" s="17" t="inlineStr">
+      <c r="M17" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>FR-INV-005</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Catalog &amp; Inventory</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Expiration Date Tracking, Shelf-Life Monitoring &amp; FEFO Clearance Alerts</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>SN-012</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>BG-010</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>BR-RUL-011</t>
+        </is>
+      </c>
+      <c r="G18" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Screen 4 (Inventory)</t>
+        </is>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
+        <is>
+          <t>src/app/inventory.tsx
+src/domain/entities/Product.ts</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>products (expiry_date)</t>
+        </is>
+      </c>
+      <c r="K18" s="15" t="inlineStr">
+        <is>
+          <t>FEFO Alert Triage &amp; Checkout Expiration Blocker Test</t>
+        </is>
+      </c>
+      <c r="L18" s="10" t="inlineStr">
+        <is>
+          <t>TC-FR-INV-005</t>
+        </is>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>FR-EXC-001</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>Exception Handling</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>Same-Day Sales Void with Automatic Stock Reversal</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>SN-004</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>BG-004</t>
         </is>
       </c>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>BR-RUL-002, BR-RUL-006</t>
         </is>
       </c>
-      <c r="G16" s="16" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="H19" s="12" t="inlineStr">
         <is>
           <t>Screen 5 (Sales History)</t>
         </is>
       </c>
-      <c r="I16" s="15" t="inlineStr">
+      <c r="I19" s="18" t="inlineStr">
         <is>
           <t>src/app/sales.tsx
 src/application/TindahanStoreService.ts</t>
         </is>
       </c>
-      <c r="J16" s="10" t="inlineStr">
+      <c r="J19" s="12" t="inlineStr">
         <is>
           <t>sales_transactions, products, monthly_sales_history</t>
         </is>
       </c>
-      <c r="K16" s="15" t="inlineStr">
+      <c r="K19" s="18" t="inlineStr">
         <is>
           <t>Atomic Transaction Unit Test</t>
         </is>
       </c>
-      <c r="L16" s="10" t="inlineStr">
+      <c r="L19" s="12" t="inlineStr">
         <is>
           <t>TC-FR-EXC-001</t>
         </is>
       </c>
-      <c r="M16" s="17" t="inlineStr">
+      <c r="M19" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>FR-EXC-002</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Exception Handling</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>Receipt-Linked Return Wizard with Quantity Capping</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>SN-004</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>BG-004</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>BR-RUL-002</t>
         </is>
       </c>
-      <c r="G17" s="16" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="H20" s="10" t="inlineStr">
         <is>
           <t>Screen 5 (Sales History)</t>
         </is>
       </c>
-      <c r="I17" s="18" t="inlineStr">
+      <c r="I20" s="15" t="inlineStr">
         <is>
           <t>src/app/sales.tsx
 src/application/TindahanStoreService.ts</t>
         </is>
       </c>
-      <c r="J17" s="12" t="inlineStr">
+      <c r="J20" s="10" t="inlineStr">
         <is>
           <t>sales_transactions</t>
         </is>
       </c>
-      <c r="K17" s="18" t="inlineStr">
+      <c r="K20" s="15" t="inlineStr">
         <is>
           <t>Boundary Value Test (Return Qty &lt;= Purchased Qty)</t>
         </is>
       </c>
-      <c r="L17" s="12" t="inlineStr">
+      <c r="L20" s="10" t="inlineStr">
         <is>
           <t>TC-FR-EXC-002</t>
         </is>
       </c>
-      <c r="M17" s="17" t="inlineStr">
+      <c r="M20" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>FR-EXC-003</t>
         </is>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>Exception Handling</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Mandatory Condition Disposition Gating (Sellable vs. Bad Order Quarantine)</t>
         </is>
       </c>
-      <c r="D18" s="10" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>SN-004</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>BG-004</t>
         </is>
       </c>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>BR-RUL-002</t>
         </is>
       </c>
-      <c r="G18" s="16" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="H21" s="12" t="inlineStr">
         <is>
           <t>Screen 5 (Sales History)</t>
         </is>
       </c>
-      <c r="I18" s="15" t="inlineStr">
+      <c r="I21" s="18" t="inlineStr">
         <is>
           <t>src/app/sales.tsx
 src/application/TindahanStoreService.ts</t>
         </is>
       </c>
-      <c r="J18" s="10" t="inlineStr">
+      <c r="J21" s="12" t="inlineStr">
         <is>
           <t>products (quarantine_stock_count), shrinkage_logs</t>
         </is>
       </c>
-      <c r="K18" s="15" t="inlineStr">
+      <c r="K21" s="18" t="inlineStr">
         <is>
           <t>Integration Test (Zero Phantom Inventory)</t>
         </is>
       </c>
-      <c r="L18" s="10" t="inlineStr">
+      <c r="L21" s="12" t="inlineStr">
         <is>
           <t>TC-FR-EXC-003</t>
         </is>
       </c>
-      <c r="M18" s="17" t="inlineStr">
+      <c r="M21" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>FR-EXC-004</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Exception Handling</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>Atomic In-Flow Product Exchange Settlement</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>SN-004</t>
         </is>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>BG-004</t>
         </is>
       </c>
-      <c r="F19" s="12" t="inlineStr">
+      <c r="F22" s="10" t="inlineStr">
         <is>
           <t>BR-RUL-002</t>
         </is>
       </c>
-      <c r="G19" s="16" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H19" s="12" t="inlineStr">
+      <c r="H22" s="10" t="inlineStr">
         <is>
           <t>Screen 5 -&gt; Screen 3</t>
         </is>
       </c>
-      <c r="I19" s="18" t="inlineStr">
+      <c r="I22" s="15" t="inlineStr">
         <is>
           <t>src/app/sales.tsx
 src/app/checkout.tsx</t>
         </is>
       </c>
-      <c r="J19" s="12" t="inlineStr">
+      <c r="J22" s="10" t="inlineStr">
         <is>
           <t>sales_transactions, products</t>
         </is>
       </c>
-      <c r="K19" s="18" t="inlineStr">
+      <c r="K22" s="15" t="inlineStr">
         <is>
           <t>End-to-End Exchange Delta Calculation Test</t>
         </is>
       </c>
-      <c r="L19" s="12" t="inlineStr">
+      <c r="L22" s="10" t="inlineStr">
         <is>
           <t>TC-FR-EXC-004</t>
         </is>
       </c>
-      <c r="M19" s="17" t="inlineStr">
+      <c r="M22" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>FR-UTG-001</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>Utang Credit Ledger</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Customer Credit Profile &amp; Credit Limit Enforcement</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>SN-005</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>BG-005</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>BR-RUL-003</t>
         </is>
       </c>
-      <c r="G20" s="16" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H20" s="10" t="inlineStr">
+      <c r="H23" s="12" t="inlineStr">
         <is>
           <t>Screen 6 -&gt; Utang</t>
         </is>
       </c>
-      <c r="I20" s="15" t="inlineStr">
+      <c r="I23" s="18" t="inlineStr">
         <is>
           <t>src/app/utang.tsx
 src/application/TindahanStoreService.ts</t>
         </is>
       </c>
-      <c r="J20" s="10" t="inlineStr">
+      <c r="J23" s="12" t="inlineStr">
         <is>
           <t>utang_customers</t>
         </is>
       </c>
-      <c r="K20" s="15" t="inlineStr">
+      <c r="K23" s="18" t="inlineStr">
         <is>
           <t>Unit Test (Credit Ceiling Validation)</t>
         </is>
       </c>
-      <c r="L20" s="10" t="inlineStr">
+      <c r="L23" s="12" t="inlineStr">
         <is>
           <t>TC-FR-UTG-001</t>
         </is>
       </c>
-      <c r="M20" s="17" t="inlineStr">
+      <c r="M23" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>FR-UTG-002</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Utang Credit Ledger</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>Checkout Direct Charge to Customer Tab &amp; Demand Imputation</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>SN-005</t>
         </is>
       </c>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>BG-005</t>
         </is>
       </c>
-      <c r="F21" s="12" t="inlineStr">
+      <c r="F24" s="10" t="inlineStr">
         <is>
           <t>BR-RUL-003</t>
         </is>
       </c>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H21" s="12" t="inlineStr">
+      <c r="H24" s="10" t="inlineStr">
         <is>
           <t>Screen 3 (Checkout)</t>
         </is>
       </c>
-      <c r="I21" s="18" t="inlineStr">
+      <c r="I24" s="15" t="inlineStr">
         <is>
           <t>src/app/checkout.tsx
 src/application/TindahanStoreService.ts</t>
         </is>
       </c>
-      <c r="J21" s="12" t="inlineStr">
+      <c r="J24" s="10" t="inlineStr">
         <is>
           <t>utang_customers, sales_transactions, monthly_sales_history</t>
         </is>
       </c>
-      <c r="K21" s="18" t="inlineStr">
+      <c r="K24" s="15" t="inlineStr">
         <is>
           <t>Atomic Split &amp; Balance Update Test</t>
         </is>
       </c>
-      <c r="L21" s="12" t="inlineStr">
+      <c r="L24" s="10" t="inlineStr">
         <is>
           <t>TC-FR-UTG-002</t>
         </is>
       </c>
-      <c r="M21" s="17" t="inlineStr">
+      <c r="M24" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>FR-UTG-003</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>Utang Credit Ledger</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>Partial &amp; Full Debt Payment Reconciliation</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>SN-005</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>BG-005</t>
         </is>
       </c>
-      <c r="F22" s="10" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>BR-RUL-003</t>
         </is>
       </c>
-      <c r="G22" s="16" t="inlineStr">
+      <c r="G25" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H22" s="10" t="inlineStr">
+      <c r="H25" s="12" t="inlineStr">
         <is>
           <t>Screen 6 -&gt; Utang</t>
         </is>
       </c>
-      <c r="I22" s="15" t="inlineStr">
+      <c r="I25" s="18" t="inlineStr">
         <is>
           <t>src/app/utang.tsx
 src/application/TindahanStoreService.ts</t>
         </is>
       </c>
-      <c r="J22" s="10" t="inlineStr">
+      <c r="J25" s="12" t="inlineStr">
         <is>
           <t>utang_customers, cash_drawer_adjustments</t>
         </is>
       </c>
-      <c r="K22" s="15" t="inlineStr">
+      <c r="K25" s="18" t="inlineStr">
         <is>
           <t>Cash Drawer Inflow &amp; Ledger Reconciliation Test</t>
         </is>
       </c>
-      <c r="L22" s="10" t="inlineStr">
+      <c r="L25" s="12" t="inlineStr">
         <is>
           <t>TC-FR-UTG-003</t>
-        </is>
-      </c>
-      <c r="M22" s="17" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>FR-UTG-004</t>
-        </is>
-      </c>
-      <c r="B23" s="18" t="inlineStr">
-        <is>
-          <t>Utang Credit Ledger</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>Customer Debt Statement Image Export</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>SN-005</t>
-        </is>
-      </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>BG-005</t>
-        </is>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
-        <is>
-          <t>BR-RUL-003</t>
-        </is>
-      </c>
-      <c r="G23" s="19" t="inlineStr">
-        <is>
-          <t>SHOULD</t>
-        </is>
-      </c>
-      <c r="H23" s="12" t="inlineStr">
-        <is>
-          <t>Screen 6 -&gt; Utang</t>
-        </is>
-      </c>
-      <c r="I23" s="18" t="inlineStr">
-        <is>
-          <t>src/app/utang.tsx (react-native-view-shot)</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="inlineStr">
-        <is>
-          <t>Local Storage / Share Sheet</t>
-        </is>
-      </c>
-      <c r="K23" s="18" t="inlineStr">
-        <is>
-          <t>Native Share Dialog Test</t>
-        </is>
-      </c>
-      <c r="L23" s="12" t="inlineStr">
-        <is>
-          <t>TC-FR-UTG-004</t>
-        </is>
-      </c>
-      <c r="M23" s="17" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>FR-FOR-001</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>Seasonal Forecast</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>Multi-Tier Historical Demand Analysis (12-23M vs 24M+ YoY)</t>
-        </is>
-      </c>
-      <c r="D24" s="10" t="inlineStr">
-        <is>
-          <t>SN-006</t>
-        </is>
-      </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>BG-006</t>
-        </is>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>BR-RUL-006</t>
-        </is>
-      </c>
-      <c r="G24" s="16" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-      <c r="H24" s="10" t="inlineStr">
-        <is>
-          <t>Screen 6 &amp; Screen 4</t>
-        </is>
-      </c>
-      <c r="I24" s="15" t="inlineStr">
-        <is>
-          <t>src/domain/strategies/SeasonalForecastEngine.ts</t>
-        </is>
-      </c>
-      <c r="J24" s="10" t="inlineStr">
-        <is>
-          <t>monthly_sales_history</t>
-        </is>
-      </c>
-      <c r="K24" s="15" t="inlineStr">
-        <is>
-          <t>Algorithmic Precision Unit Tests</t>
-        </is>
-      </c>
-      <c r="L24" s="10" t="inlineStr">
-        <is>
-          <t>TC-FR-FOR-001</t>
-        </is>
-      </c>
-      <c r="M24" s="17" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>FR-FOR-002</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="inlineStr">
-        <is>
-          <t>Seasonal Forecast</t>
-        </is>
-      </c>
-      <c r="C25" s="18" t="inlineStr">
-        <is>
-          <t>Demand Uncensoring for Stockout Days (Availability Factor)</t>
-        </is>
-      </c>
-      <c r="D25" s="12" t="inlineStr">
-        <is>
-          <t>SN-006</t>
-        </is>
-      </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>BG-006</t>
-        </is>
-      </c>
-      <c r="F25" s="12" t="inlineStr">
-        <is>
-          <t>BR-RUL-006</t>
-        </is>
-      </c>
-      <c r="G25" s="16" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-      <c r="H25" s="12" t="inlineStr">
-        <is>
-          <t>Screen 6 &amp; Screen 4</t>
-        </is>
-      </c>
-      <c r="I25" s="18" t="inlineStr">
-        <is>
-          <t>src/domain/strategies/SeasonalForecastEngine.ts</t>
-        </is>
-      </c>
-      <c r="J25" s="12" t="inlineStr">
-        <is>
-          <t>monthly_sales_history (out_of_stock_days)</t>
-        </is>
-      </c>
-      <c r="K25" s="18" t="inlineStr">
-        <is>
-          <t>Mathematical Model Unit Tests</t>
-        </is>
-      </c>
-      <c r="L25" s="12" t="inlineStr">
-        <is>
-          <t>TC-FR-FOR-002</t>
         </is>
       </c>
       <c r="M25" s="17" t="inlineStr">
@@ -3018,62 +3056,62 @@
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>FR-FOR-003</t>
+          <t>FR-UTG-004</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>Seasonal Forecast</t>
+          <t>Utang Credit Ledger</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>Anomaly Filtering (One-Time Bulk Orders &amp; Voids Exclusion)</t>
+          <t>Customer Debt Statement Image Export</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>SN-006</t>
+          <t>SN-005</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>BG-006</t>
+          <t>BG-005</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
         <is>
-          <t>BR-RUL-006</t>
-        </is>
-      </c>
-      <c r="G26" s="16" t="inlineStr">
-        <is>
-          <t>MUST</t>
+          <t>BR-RUL-003</t>
+        </is>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
         </is>
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>Screen 6 &amp; Screen 4</t>
+          <t>Screen 6 -&gt; Utang</t>
         </is>
       </c>
       <c r="I26" s="15" t="inlineStr">
         <is>
-          <t>src/domain/strategies/SeasonalForecastEngine.ts</t>
+          <t>src/app/utang.tsx (react-native-view-shot)</t>
         </is>
       </c>
       <c r="J26" s="10" t="inlineStr">
         <is>
-          <t>sales_transactions (is_one_time_bulk_order)</t>
+          <t>Local Storage / Share Sheet</t>
         </is>
       </c>
       <c r="K26" s="15" t="inlineStr">
         <is>
-          <t>Regression Unit Tests (Fiesta Outlier Removal)</t>
+          <t>Native Share Dialog Test</t>
         </is>
       </c>
       <c r="L26" s="10" t="inlineStr">
         <is>
-          <t>TC-FR-FOR-003</t>
+          <t>TC-FR-UTG-004</t>
         </is>
       </c>
       <c r="M26" s="17" t="inlineStr">
@@ -3085,264 +3123,264 @@
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
+          <t>FR-FOR-001</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Seasonal Forecast</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Multi-Tier Historical Demand Analysis (12-23M vs 24M+ YoY)</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>SN-006</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>BG-006</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>BR-RUL-006</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>Screen 6 &amp; Screen 4</t>
+        </is>
+      </c>
+      <c r="I27" s="18" t="inlineStr">
+        <is>
+          <t>src/domain/strategies/SeasonalForecastEngine.ts</t>
+        </is>
+      </c>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>monthly_sales_history</t>
+        </is>
+      </c>
+      <c r="K27" s="18" t="inlineStr">
+        <is>
+          <t>Algorithmic Precision Unit Tests</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>TC-FR-FOR-001</t>
+        </is>
+      </c>
+      <c r="M27" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>FR-FOR-002</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>Seasonal Forecast</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>Demand Uncensoring for Stockout Days (Availability Factor)</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>SN-006</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>BG-006</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>BR-RUL-006</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>Screen 6 &amp; Screen 4</t>
+        </is>
+      </c>
+      <c r="I28" s="15" t="inlineStr">
+        <is>
+          <t>src/domain/strategies/SeasonalForecastEngine.ts</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>monthly_sales_history (out_of_stock_days)</t>
+        </is>
+      </c>
+      <c r="K28" s="15" t="inlineStr">
+        <is>
+          <t>Mathematical Model Unit Tests</t>
+        </is>
+      </c>
+      <c r="L28" s="10" t="inlineStr">
+        <is>
+          <t>TC-FR-FOR-002</t>
+        </is>
+      </c>
+      <c r="M28" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>FR-FOR-003</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>Seasonal Forecast</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>Anomaly Filtering (One-Time Bulk Orders &amp; Voids Exclusion)</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>SN-006</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>BG-006</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>BR-RUL-006</t>
+        </is>
+      </c>
+      <c r="G29" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>Screen 6 &amp; Screen 4</t>
+        </is>
+      </c>
+      <c r="I29" s="18" t="inlineStr">
+        <is>
+          <t>src/domain/strategies/SeasonalForecastEngine.ts</t>
+        </is>
+      </c>
+      <c r="J29" s="12" t="inlineStr">
+        <is>
+          <t>sales_transactions (is_one_time_bulk_order)</t>
+        </is>
+      </c>
+      <c r="K29" s="18" t="inlineStr">
+        <is>
+          <t>Regression Unit Tests (Fiesta Outlier Removal)</t>
+        </is>
+      </c>
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>TC-FR-FOR-003</t>
+        </is>
+      </c>
+      <c r="M29" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
           <t>FR-FOR-004</t>
         </is>
       </c>
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Seasonal Forecast</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>Plain-Language Restock Recommendations &amp; Wholesale Capital Budgeting</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>SN-006</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>BG-006</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="F30" s="10" t="inlineStr">
         <is>
           <t>BR-RUL-006</t>
         </is>
       </c>
-      <c r="G27" s="16" t="inlineStr">
+      <c r="G30" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H27" s="12" t="inlineStr">
+      <c r="H30" s="10" t="inlineStr">
         <is>
           <t>Screen 4 &amp; Screen 6</t>
         </is>
       </c>
-      <c r="I27" s="18" t="inlineStr">
+      <c r="I30" s="15" t="inlineStr">
         <is>
           <t>src/app/inventory.tsx
 src/domain/strategies/SeasonalForecastEngine.ts</t>
         </is>
       </c>
-      <c r="J27" s="12" t="inlineStr">
+      <c r="J30" s="10" t="inlineStr">
         <is>
           <t>store_settings (wholesale_budget_php)</t>
         </is>
       </c>
-      <c r="K27" s="18" t="inlineStr">
+      <c r="K30" s="15" t="inlineStr">
         <is>
           <t>Integration Test (Budget Pro-rating)</t>
         </is>
       </c>
-      <c r="L27" s="12" t="inlineStr">
+      <c r="L30" s="10" t="inlineStr">
         <is>
           <t>TC-FR-FOR-004</t>
-        </is>
-      </c>
-      <c r="M27" s="17" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>FR-FOR-005</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>Seasonal Forecast</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>1-Tap Wholesale Shopping List Image Export</t>
-        </is>
-      </c>
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>SN-006</t>
-        </is>
-      </c>
-      <c r="E28" s="10" t="inlineStr">
-        <is>
-          <t>BG-006</t>
-        </is>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
-        <is>
-          <t>BR-RUL-006</t>
-        </is>
-      </c>
-      <c r="G28" s="19" t="inlineStr">
-        <is>
-          <t>SHOULD</t>
-        </is>
-      </c>
-      <c r="H28" s="10" t="inlineStr">
-        <is>
-          <t>Screen 6 (Sales Reports)</t>
-        </is>
-      </c>
-      <c r="I28" s="15" t="inlineStr">
-        <is>
-          <t>src/app/more.tsx (react-native-view-shot)</t>
-        </is>
-      </c>
-      <c r="J28" s="10" t="inlineStr">
-        <is>
-          <t>Local Storage / Share Sheet</t>
-        </is>
-      </c>
-      <c r="K28" s="15" t="inlineStr">
-        <is>
-          <t>Native Share Intent Test</t>
-        </is>
-      </c>
-      <c r="L28" s="10" t="inlineStr">
-        <is>
-          <t>TC-FR-FOR-005</t>
-        </is>
-      </c>
-      <c r="M28" s="17" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>FR-CSH-001</t>
-        </is>
-      </c>
-      <c r="B29" s="18" t="inlineStr">
-        <is>
-          <t>Cash Drawer Operations</t>
-        </is>
-      </c>
-      <c r="C29" s="18" t="inlineStr">
-        <is>
-          <t>Cash Drawer Float &amp; Paid-In / Paid-Out Logging</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>SN-002</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>BG-002</t>
-        </is>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>BR-RUL-004</t>
-        </is>
-      </c>
-      <c r="G29" s="16" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-      <c r="H29" s="12" t="inlineStr">
-        <is>
-          <t>Screen 6 -&gt; Drawer</t>
-        </is>
-      </c>
-      <c r="I29" s="18" t="inlineStr">
-        <is>
-          <t>src/application/TindahanStoreService.ts</t>
-        </is>
-      </c>
-      <c r="J29" s="12" t="inlineStr">
-        <is>
-          <t>cash_drawer_adjustments</t>
-        </is>
-      </c>
-      <c r="K29" s="18" t="inlineStr">
-        <is>
-          <t>Cash Ledger Balance Test</t>
-        </is>
-      </c>
-      <c r="L29" s="12" t="inlineStr">
-        <is>
-          <t>TC-FR-CSH-001</t>
-        </is>
-      </c>
-      <c r="M29" s="17" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>FR-CSH-002</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="inlineStr">
-        <is>
-          <t>Cash Drawer Operations</t>
-        </is>
-      </c>
-      <c r="C30" s="15" t="inlineStr">
-        <is>
-          <t>End-of-Day Cash Drawer Reconciliation &amp; Variance Calculator</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>SN-002</t>
-        </is>
-      </c>
-      <c r="E30" s="10" t="inlineStr">
-        <is>
-          <t>BG-002</t>
-        </is>
-      </c>
-      <c r="F30" s="10" t="inlineStr">
-        <is>
-          <t>BR-RUL-004</t>
-        </is>
-      </c>
-      <c r="G30" s="16" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-      <c r="H30" s="10" t="inlineStr">
-        <is>
-          <t>Screen 6 -&gt; Drawer</t>
-        </is>
-      </c>
-      <c r="I30" s="15" t="inlineStr">
-        <is>
-          <t>src/application/TindahanStoreService.ts</t>
-        </is>
-      </c>
-      <c r="J30" s="10" t="inlineStr">
-        <is>
-          <t>cash_drawer_adjustments, sales_transactions</t>
-        </is>
-      </c>
-      <c r="K30" s="15" t="inlineStr">
-        <is>
-          <t>Daily Cash Balancing Calculation Test</t>
-        </is>
-      </c>
-      <c r="L30" s="10" t="inlineStr">
-        <is>
-          <t>TC-FR-CSH-002</t>
         </is>
       </c>
       <c r="M30" s="17" t="inlineStr">
@@ -3354,202 +3392,539 @@
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="12" t="inlineStr">
         <is>
+          <t>FR-FOR-005</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>Seasonal Forecast</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>1-Tap Wholesale Shopping List Image Export</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>SN-006</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>BG-006</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>BR-RUL-006</t>
+        </is>
+      </c>
+      <c r="G31" s="19" t="inlineStr">
+        <is>
+          <t>SHOULD</t>
+        </is>
+      </c>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>Screen 6 (Sales Reports)</t>
+        </is>
+      </c>
+      <c r="I31" s="18" t="inlineStr">
+        <is>
+          <t>src/app/more.tsx (react-native-view-shot)</t>
+        </is>
+      </c>
+      <c r="J31" s="12" t="inlineStr">
+        <is>
+          <t>Local Storage / Share Sheet</t>
+        </is>
+      </c>
+      <c r="K31" s="18" t="inlineStr">
+        <is>
+          <t>Native Share Intent Test</t>
+        </is>
+      </c>
+      <c r="L31" s="12" t="inlineStr">
+        <is>
+          <t>TC-FR-FOR-005</t>
+        </is>
+      </c>
+      <c r="M31" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>FR-CSH-001</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>Cash Drawer Operations</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>Cash Drawer Float &amp; Paid-In / Paid-Out Logging</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>SN-002</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>BG-002</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>BR-RUL-004</t>
+        </is>
+      </c>
+      <c r="G32" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>Screen 6 -&gt; Drawer</t>
+        </is>
+      </c>
+      <c r="I32" s="15" t="inlineStr">
+        <is>
+          <t>src/application/TindahanStoreService.ts</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t>cash_drawer_adjustments</t>
+        </is>
+      </c>
+      <c r="K32" s="15" t="inlineStr">
+        <is>
+          <t>Cash Ledger Balance Test</t>
+        </is>
+      </c>
+      <c r="L32" s="10" t="inlineStr">
+        <is>
+          <t>TC-FR-CSH-001</t>
+        </is>
+      </c>
+      <c r="M32" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>FR-CSH-002</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>Cash Drawer Operations</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>End-of-Day Cash Drawer Reconciliation &amp; Variance Calculator</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>SN-002</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>BG-002</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>BR-RUL-004</t>
+        </is>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>Screen 6 -&gt; Drawer</t>
+        </is>
+      </c>
+      <c r="I33" s="18" t="inlineStr">
+        <is>
+          <t>src/application/TindahanStoreService.ts</t>
+        </is>
+      </c>
+      <c r="J33" s="12" t="inlineStr">
+        <is>
+          <t>cash_drawer_adjustments, sales_transactions</t>
+        </is>
+      </c>
+      <c r="K33" s="18" t="inlineStr">
+        <is>
+          <t>Daily Cash Balancing Calculation Test</t>
+        </is>
+      </c>
+      <c r="L33" s="12" t="inlineStr">
+        <is>
+          <t>TC-FR-CSH-002</t>
+        </is>
+      </c>
+      <c r="M33" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
           <t>FR-SET-001</t>
         </is>
       </c>
-      <c r="B31" s="18" t="inlineStr">
+      <c r="B34" s="15" t="inlineStr">
         <is>
           <t>Settings &amp; Preferences</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
-        <is>
-          <t>Store Identity &amp; Operational Branding Preferences</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>SN-007</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="inlineStr">
-        <is>
-          <t>BG-007</t>
-        </is>
-      </c>
-      <c r="F31" s="12" t="inlineStr">
-        <is>
-          <t>BR-RUL-001</t>
-        </is>
-      </c>
-      <c r="G31" s="16" t="inlineStr">
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>Store Identity, Bilingual Localization &amp; Operational Preferences</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>SN-007, SN-010</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>BG-001, BG-007</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>BR-RUL-009</t>
+        </is>
+      </c>
+      <c r="G34" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H31" s="12" t="inlineStr">
+      <c r="H34" s="10" t="inlineStr">
         <is>
           <t>Screen 7 (Settings)</t>
         </is>
       </c>
-      <c r="I31" s="18" t="inlineStr">
+      <c r="I34" s="15" t="inlineStr">
         <is>
           <t>src/app/settings.tsx
 src/application/TindahanStoreService.ts</t>
         </is>
       </c>
-      <c r="J31" s="12" t="inlineStr">
-        <is>
-          <t>store_settings</t>
-        </is>
-      </c>
-      <c r="K31" s="18" t="inlineStr">
-        <is>
-          <t>CRUD Persistence Unit Test</t>
-        </is>
-      </c>
-      <c r="L31" s="12" t="inlineStr">
+      <c r="J34" s="10" t="inlineStr">
+        <is>
+          <t>store_settings, KeyValueStorage</t>
+        </is>
+      </c>
+      <c r="K34" s="15" t="inlineStr">
+        <is>
+          <t>CRUD &amp; Cold-Boot Storage Precedence Test</t>
+        </is>
+      </c>
+      <c r="L34" s="10" t="inlineStr">
         <is>
           <t>TC-FR-SET-001</t>
         </is>
       </c>
-      <c r="M31" s="17" t="inlineStr">
+      <c r="M34" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>FR-SET-002</t>
         </is>
       </c>
-      <c r="B32" s="15" t="inlineStr">
+      <c r="B35" s="18" t="inlineStr">
         <is>
           <t>Settings &amp; Preferences</t>
         </is>
       </c>
-      <c r="C32" s="15" t="inlineStr">
-        <is>
-          <t>Seasonal Calendar Configuration (School Opening, Town Fiesta)</t>
-        </is>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>Seasonal Calendar Configuration (School Opening &amp; Wholesale Budget)</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>SN-006</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>BG-006</t>
         </is>
       </c>
-      <c r="F32" s="10" t="inlineStr">
+      <c r="F35" s="12" t="inlineStr">
         <is>
           <t>BR-RUL-006</t>
         </is>
       </c>
-      <c r="G32" s="16" t="inlineStr">
+      <c r="G35" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H32" s="10" t="inlineStr">
+      <c r="H35" s="12" t="inlineStr">
         <is>
           <t>Screen 7 (Settings)</t>
         </is>
       </c>
-      <c r="I32" s="15" t="inlineStr">
+      <c r="I35" s="18" t="inlineStr">
         <is>
           <t>src/app/settings.tsx
 src/domain/strategies/SeasonalForecastEngine.ts</t>
         </is>
       </c>
-      <c r="J32" s="10" t="inlineStr">
+      <c r="J35" s="12" t="inlineStr">
         <is>
           <t>store_settings</t>
         </is>
       </c>
-      <c r="K32" s="15" t="inlineStr">
+      <c r="K35" s="18" t="inlineStr">
         <is>
           <t>Calendar Trigger Integration Test</t>
         </is>
       </c>
-      <c r="L32" s="10" t="inlineStr">
+      <c r="L35" s="12" t="inlineStr">
         <is>
           <t>TC-FR-SET-002</t>
         </is>
       </c>
-      <c r="M32" s="17" t="inlineStr">
+      <c r="M35" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="12" t="inlineStr">
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>FR-SET-003</t>
         </is>
       </c>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="B36" s="15" t="inlineStr">
         <is>
           <t>Settings &amp; Preferences</t>
         </is>
       </c>
-      <c r="C33" s="18" t="inlineStr">
+      <c r="C36" s="15" t="inlineStr">
         <is>
           <t>Local SQLite Database Export &amp; Recovery Import</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>SN-007</t>
         </is>
       </c>
-      <c r="E33" s="12" t="inlineStr">
+      <c r="E36" s="10" t="inlineStr">
         <is>
           <t>BG-007</t>
         </is>
       </c>
-      <c r="F33" s="12" t="inlineStr">
+      <c r="F36" s="10" t="inlineStr">
         <is>
           <t>BR-RUL-001</t>
         </is>
       </c>
-      <c r="G33" s="16" t="inlineStr">
+      <c r="G36" s="16" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
       </c>
-      <c r="H33" s="12" t="inlineStr">
+      <c r="H36" s="10" t="inlineStr">
         <is>
           <t>Screen 7 (Settings)</t>
         </is>
       </c>
-      <c r="I33" s="18" t="inlineStr">
+      <c r="I36" s="15" t="inlineStr">
         <is>
           <t>src/app/settings.tsx
 src/infrastructure/database/SqliteDatabase.ts</t>
         </is>
       </c>
-      <c r="J33" s="12" t="inlineStr">
+      <c r="J36" s="10" t="inlineStr">
         <is>
           <t>FileSystem (tindahan_pos_v3.db)</t>
         </is>
       </c>
-      <c r="K33" s="18" t="inlineStr">
+      <c r="K36" s="15" t="inlineStr">
         <is>
           <t>Database Backup/Restore Integrity Test</t>
         </is>
       </c>
-      <c r="L33" s="12" t="inlineStr">
+      <c r="L36" s="10" t="inlineStr">
         <is>
           <t>TC-FR-SET-003</t>
         </is>
       </c>
-      <c r="M33" s="17" t="inlineStr">
+      <c r="M36" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>FR-SEC-001</t>
+        </is>
+      </c>
+      <c r="B37" s="18" t="inlineStr">
+        <is>
+          <t>Settings &amp; Security</t>
+        </is>
+      </c>
+      <c r="C37" s="18" t="inlineStr">
+        <is>
+          <t>Owner Master PIN &amp; Relief Cashier Operational Access Control</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>SN-011</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>BG-009</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>BR-RUL-010</t>
+        </is>
+      </c>
+      <c r="G37" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>Screen 7 &amp; Global Modal</t>
+        </is>
+      </c>
+      <c r="I37" s="18" t="inlineStr">
+        <is>
+          <t>src/app/settings.tsx
+src/infrastructure/storage/KeyValueStorage.ts</t>
+        </is>
+      </c>
+      <c r="J37" s="12" t="inlineStr">
+        <is>
+          <t>store_settings, KeyValueStorage</t>
+        </is>
+      </c>
+      <c r="K37" s="18" t="inlineStr">
+        <is>
+          <t>Cashier Role Boundary &amp; 5-Try Lockout Test</t>
+        </is>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>TC-FR-SEC-001</t>
+        </is>
+      </c>
+      <c r="M37" s="17" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>FR-SAL-001</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>Sales &amp; Profit Intelligence</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>Sales History, Gross Profit (Tubo / Markup) Intelligence &amp; Z-Reading</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>SN-009</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>BG-001, BG-002</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>BR-RUL-008</t>
+        </is>
+      </c>
+      <c r="G38" s="16" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+      <c r="H38" s="10" t="inlineStr">
+        <is>
+          <t>Screen 5 (Sales History)</t>
+        </is>
+      </c>
+      <c r="I38" s="15" t="inlineStr">
+        <is>
+          <t>src/app/sales.tsx
+src/presentation/hooks/useTindahanStore.ts</t>
+        </is>
+      </c>
+      <c r="J38" s="10" t="inlineStr">
+        <is>
+          <t>sales_transactions, products</t>
+        </is>
+      </c>
+      <c r="K38" s="15" t="inlineStr">
+        <is>
+          <t>Unit &amp; UI Test (Snapshot COGS, Tubo Formula, Privacy Eye Mask)</t>
+        </is>
+      </c>
+      <c r="L38" s="10" t="inlineStr">
+        <is>
+          <t>TC-FR-SAL-001</t>
+        </is>
+      </c>
+      <c r="M38" s="17" t="inlineStr">
         <is>
           <t>VERIFIED</t>
         </is>
@@ -3566,13 +3941,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
@@ -4350,27 +4725,28 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Bilingual Localization (English &amp; Filipino)</t>
+          <t>Multi-Dialect Localization (English, Filipino, Taglish) &amp; Storage Precedence</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>100% dictionary string parity</t>
+          <t>100% dictionary string parity across en/fil/taglish with storage precedence</t>
         </is>
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>src/presentation/localization/i18n.ts with zero-restart toggle</t>
+          <t>src/presentation/localization/i18n.ts with KeyValueStorage precedence on cold boot</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>src/presentation/localization/i18n.ts</t>
+          <t>src/presentation/localization/i18n.ts
+src/infrastructure/storage/KeyValueStorage.ts</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
         <is>
-          <t>Jest Translation Key Parity Linter</t>
+          <t>Jest Translation Key Parity &amp; Hydration Test</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
@@ -4575,42 +4951,42 @@
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>NFR-ARC-001</t>
+          <t>NFR-SEC-005</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Maintainability</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>Clean Architecture &amp; Layer Decoupling</t>
+          <t>Counter Profit Privacy Masking (Owner Tubo Obfuscation)</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Domain has 0 React/SQLite imports</t>
+          <t>100% profit/markup masked with •••••• in &lt;= 16ms</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>Strict separation: Domain, Application, Infrastructure, Presentation</t>
+          <t>Owner privacy toggle button obfuscating sensitive wholesale margins from counter onlookers</t>
         </is>
       </c>
       <c r="F22" s="15" t="inlineStr">
         <is>
-          <t>Whole Repository</t>
+          <t>src/app/sales.tsx</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>ESLint Dependency Boundary Rules</t>
+          <t>Automated UI Privacy Mask Verification Suite</t>
         </is>
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>TC-NFR-ARC-001</t>
+          <t>TC-NFR-SEC-005</t>
         </is>
       </c>
       <c r="I22" s="17" t="inlineStr">
@@ -4622,42 +4998,42 @@
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>NFR-ARC-002</t>
+          <t>NFR-SEC-006</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Maintainability</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Zero Floating-Point Penny Drift</t>
+          <t>Owner Master PIN Cryptographic Hash &amp; Brute-Force Rate Limiting</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Exact integer centavo math</t>
+          <t>Salted SHA-256 hash; 5-attempt / 300s lockout</t>
         </is>
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>Money Value Object; calculations in centavos (* 100)</t>
+          <t>Salted cryptographic PIN hash in sandboxed storage with persistent lockout timer</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>src/domain/value-objects/Money.ts</t>
+          <t>src/infrastructure/storage/KeyValueStorage.ts</t>
         </is>
       </c>
       <c r="G23" s="18" t="inlineStr">
         <is>
-          <t>100,000 Randomized Split Calculations Test</t>
+          <t>Jest PIN Security Suite &amp; Reboot Persistence Test</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
         <is>
-          <t>TC-NFR-ARC-002</t>
+          <t>TC-NFR-SEC-006</t>
         </is>
       </c>
       <c r="I23" s="17" t="inlineStr">
@@ -4669,7 +5045,7 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>NFR-ARC-003</t>
+          <t>NFR-ARC-001</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -4679,17 +5055,17 @@
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>100% Strict TypeScript Compilation</t>
+          <t>Clean Architecture &amp; Layer Decoupling</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>0 compilation errors / warnings</t>
+          <t>Domain has 0 React/SQLite imports</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>Strict compiler options (noImplicitAny, strictNullChecks)</t>
+          <t>Strict separation: Domain, Application, Infrastructure, Presentation</t>
         </is>
       </c>
       <c r="F24" s="15" t="inlineStr">
@@ -4699,12 +5075,12 @@
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>npx tsc --noEmit Command Verification</t>
+          <t>ESLint Dependency Boundary Rules</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>TC-NFR-ARC-003</t>
+          <t>TC-NFR-ARC-001</t>
         </is>
       </c>
       <c r="I24" s="17" t="inlineStr">
@@ -4716,42 +5092,42 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>NFR-ENV-001</t>
+          <t>NFR-ARC-002</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Environmental</t>
+          <t>Maintainability</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>Budget Mobile Hardware Compatibility</t>
+          <t>Zero Floating-Point Penny Drift</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Android 10+ with 2GB RAM</t>
+          <t>Exact integer centavo math</t>
         </is>
       </c>
       <c r="E25" s="18" t="inlineStr">
         <is>
-          <t>Compiled with Hermes JavaScript Engine and lightweight asset pipeline</t>
+          <t>Money Value Object; calculations in centavos (* 100)</t>
         </is>
       </c>
       <c r="F25" s="18" t="inlineStr">
         <is>
-          <t>app.json, package.json</t>
+          <t>src/domain/value-objects/Money.ts</t>
         </is>
       </c>
       <c r="G25" s="18" t="inlineStr">
         <is>
-          <t>Redmi 9A Reference Hardware Deployment</t>
+          <t>100,000 Randomized Split Calculations Test</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">
         <is>
-          <t>TC-NFR-ENV-001</t>
+          <t>TC-NFR-ARC-002</t>
         </is>
       </c>
       <c r="I25" s="17" t="inlineStr">
@@ -4763,45 +5139,186 @@
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="10" t="inlineStr">
         <is>
+          <t>NFR-ARC-003</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Maintainability</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>100% Strict TypeScript Compilation</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>0 compilation errors / warnings</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>Strict compiler options (noImplicitAny, strictNullChecks)</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>Whole Repository</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr">
+        <is>
+          <t>npx tsc --noEmit Command Verification</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>TC-NFR-ARC-003</t>
+        </is>
+      </c>
+      <c r="I26" s="17" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>NFR-ENV-001</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Budget Mobile Hardware Compatibility</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Android 10+ with 2GB RAM</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Compiled with Hermes JavaScript Engine and lightweight asset pipeline</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>app.json, package.json</t>
+        </is>
+      </c>
+      <c r="G27" s="18" t="inlineStr">
+        <is>
+          <t>Redmi 9A Reference Hardware Deployment</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>TC-NFR-ENV-001</t>
+        </is>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
           <t>NFR-ENV-002</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>Environmental</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>Tropical Ambient Thermal &amp; Battery Management</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>Camera sleep at 45s; &lt;= 8% drain/hr</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>Auto-sleep inactivity timer on camera viewfinder</t>
         </is>
       </c>
-      <c r="F26" s="15" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>src/presentation/components/BarcodeScannerViewfinder.tsx</t>
         </is>
       </c>
-      <c r="G26" s="15" t="inlineStr">
+      <c r="G28" s="15" t="inlineStr">
         <is>
           <t>Thermal Chamber &amp; Battery Profiling (35°C)</t>
         </is>
       </c>
-      <c r="H26" s="10" t="inlineStr">
+      <c r="H28" s="10" t="inlineStr">
         <is>
           <t>TC-NFR-ENV-002</t>
         </is>
       </c>
-      <c r="I26" s="17" t="inlineStr">
+      <c r="I28" s="17" t="inlineStr">
+        <is>
+          <t>COMPLIANT</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>NFR-ENV-003</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Environmental</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>Extended Brownout Battery Saver &amp; AMOLED True-Black Theme</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>&gt;= 35% display power reduction on OLED/AMOLED</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>AMOLED true-black (#000000) theme tokens for extended battery runtime during 8-12h brownouts</t>
+        </is>
+      </c>
+      <c r="F29" s="18" t="inlineStr">
+        <is>
+          <t>src/constants/theme.ts</t>
+        </is>
+      </c>
+      <c r="G29" s="18" t="inlineStr">
+        <is>
+          <t>Android batterystats 2-Hour POS Profiling</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>TC-NFR-ENV-003</t>
+        </is>
+      </c>
+      <c r="I29" s="17" t="inlineStr">
         <is>
           <t>COMPLIANT</t>
         </is>
@@ -4818,14 +5335,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
     <col width="41" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
@@ -4909,7 +5426,7 @@
           <t>NFR-PERF-002, NFR-USE-001, NFR-USE-005</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="17" t="inlineStr">
         <is>
           <t>FULFILLED</t>
         </is>
@@ -4951,7 +5468,7 @@
           <t>NFR-ARC-002, NFR-USE-001</t>
         </is>
       </c>
-      <c r="H3" s="12" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>FULFILLED</t>
         </is>
@@ -4993,7 +5510,7 @@
           <t>NFR-SEC-004, NFR-ARC-002</t>
         </is>
       </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>FULFILLED</t>
         </is>
@@ -5035,7 +5552,7 @@
           <t>NFR-REL-002, NFR-SEC-004</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>FULFILLED</t>
         </is>
@@ -5077,7 +5594,7 @@
           <t>NFR-SEC-002, NFR-USE-006</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
         <is>
           <t>FULFILLED</t>
         </is>
@@ -5119,7 +5636,7 @@
           <t>NFR-PERF-003, NFR-ARC-001</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>FULFILLED</t>
         </is>
@@ -5161,7 +5678,301 @@
           <t>NFR-REL-001, NFR-REL-002, NFR-ENV-001</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="H8" s="17" t="inlineStr">
+        <is>
+          <t>FULFILLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>SN-008</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Store Owner / Relief Cashier</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Park/hold active customer baskets with customer names/notes ("Stock" Basket Queue) without losing cart items during counter interruptions or phone restarts.</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Customers pause checkout to grab forgotten items ("sandali lang may nakalimutan ako"), blocking the line for next paying customers.</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>BG-008</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>FR-POS-005</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>NFR-REL-002, NFR-USE-001</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>FULFILLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>SN-009</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Store Owner</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Monitor gross profit (tubo) and markup percentage in real time across transactions and daily periods, with immediate privacy masking from counter onlookers.</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Store owners need visibility into whether sales meet margin targets, while shielding actual wholesale costs and profit margins from customers standing at counter.</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>BG-001, BG-002</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>FR-SAL-001</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>NFR-SEC-005, NFR-ARC-002</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>FULFILLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>SN-010</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Store Owner &amp; Relief Cashier</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>Toggle and permanently persist the application language (English, Filipino, Taglish) across reboots and screen navigations.</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Relief cashiers and older store owners prefer vernacular Tagalog/Taglish labels (Tindahan, Singilin, Tubo, Talaan) without reverting to English on restart.</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>BG-001, BG-007</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>FR-SET-001</t>
+        </is>
+      </c>
+      <c r="G11" s="18" t="inlineStr">
+        <is>
+          <t>NFR-USE-006</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>FULFILLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>SN-011</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Store Owner (Juan/Maria)</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Entrust store operations to a family member or relief cashier (tindera) without risking price tampering, theft, or profit leaks.</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Owners need temporary leave from counter; untrusted access leads to price alterations, shrinkage concealment, and exposed profit margins.</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>BG-009</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>FR-SEC-001</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>NFR-SEC-006</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>FULFILLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>SN-012</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Store Owner (Juan/Maria)</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Track expiration dates for dairy, bread, and canned goods to avoid selling expired items and prevent unsellable spoilage loss.</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Expired goods lead to direct capital loss, customer health risks, and community reputation loss if sold unintentionally.</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>BG-010</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>FR-INV-005</t>
+        </is>
+      </c>
+      <c r="G13" s="18" t="inlineStr">
+        <is>
+          <t>NFR-USE-004</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>FULFILLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>SN-013</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Suki Customer &amp; Store Owner</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Provide physical printed receipt slips via cheap Bluetooth thermal printers for customers who lack smartphones or request paper proof.</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Elderly customers and market shoppers require physical paper slips; handwriting paper receipts slows counter lines.</t>
+        </is>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>BG-011</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>FR-TND-006</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>NFR-PERF-004, NFR-USE-001</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>FULFILLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>SN-014</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Store Owner &amp; Suki Customer</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>Accept and verify cashless GCash/Maya QR Ph payments with reference number logging and optional convenience surcharge to protect cash flow.</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Cashless payments without reference logging lead to screenshot scams and unverified transfers, while merchant cashout fees eat retail margins.</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>BG-012</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>FR-TND-007</t>
+        </is>
+      </c>
+      <c r="G15" s="18" t="inlineStr">
+        <is>
+          <t>NFR-ARC-002, NFR-SEC-004</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
         <is>
           <t>FULFILLED</t>
         </is>

</xml_diff>